<commit_message>
Updated JMP to expand upstream discussion
</commit_message>
<xml_diff>
--- a/papers.xlsx
+++ b/papers.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10118"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29628"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/grady/Documents/personal-website/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Grady\Documents\website\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FFFE5801-38DA-0F4C-B9FB-59C9FD5C7A92}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{63D632C7-5A11-47B7-A86C-B6592BAFD643}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="660" windowWidth="30240" windowHeight="17720" xr2:uid="{97D96D2E-9D3E-43F7-890C-EE13786D0DA2}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="38620" windowHeight="21100" xr2:uid="{97D96D2E-9D3E-43F7-890C-EE13786D0DA2}"/>
   </bookViews>
   <sheets>
     <sheet name="Working Papers" sheetId="1" r:id="rId1"/>
@@ -52,12 +52,6 @@
     <t>Abstract</t>
   </si>
   <si>
-    <t>&lt;b&gt;Job Market Paper&lt;/b&gt;</t>
-  </si>
-  <si>
-    <t>with Michael Walker, Nick Shankar, Edward Miguel and Dennis Egger</t>
-  </si>
-  <si>
     <t>Using satellites and phones to evaluate and promote agricultural technology adoption: Evidence from smallholder farms in India</t>
   </si>
   <si>
@@ -128,9 +122,6 @@
     <t>Risk Aversion and Barriers to Firm Growth: Experimental Evidence from Small Retailers</t>
   </si>
   <si>
-    <t>Firms in low and middle-income economies often grow slowly. This paper examines whether firm risk aversion prevents risk taking necessary to grow. While economists tend to model firms as risk neutral, I posit that this assumption is unlikely to hold for the modal developing country firm, which is owner-operated, so that uncertain investments may directly threaten owners’ consumption. I develop a model that shows how risk aversion can reduce firms’ willingness to experiment with new technologies, impeding investment and growth. I test the model’s predictions within the context of retail firms’ decision to adopt and sell a new consumer product using two field experiments with over 1,200 Kenyan firms. First, offering firms an insurance contract that creates a mean-preserving contraction of profits increases new product adoption by 50\%. Effects are concentrated among firms whose owners exhibit higher levels of risk aversion. Second, temporarily inducing firms to try selling a new product with a supplier returns policy leads to a 70\% increase in stock purchases after the intervention ends. Third, consistent with bandit models of learning, experimentally increasing the continuation value of learning increases adoption by 80\%. These persistent effects arise through a reduction in the variance of beliefs, rather than through changes in mean beliefs. These results show that a feature inherent to developing country environments -- small firms in the presence of missing financial markets -- itself creates a barrier to firm innovation and growth.</t>
-  </si>
-  <si>
     <t>The Long-run Effects of Unconditional Cash Transfers: Evidence from the Kenya General Equilibrium Study</t>
   </si>
   <si>
@@ -144,6 +135,15 @@
   </si>
   <si>
     <t xml:space="preserve">We estimate the impacts of large-scale unconditional cash transfers on child survival. One-time transfers of USD 1000 were provided to over 10,500 poor households across 653 randomized villages in Kenya. We collected census data on over 100,000 births, including on mortality and cause of death, and detailed data on health behaviors. Unconditional cash transfers (accounting for spillovers) lead to 48\% fewer infant deaths before age one and 45\% fewer child deaths before age five. These improvements appear to arise from better maternal health and nutrition, a 53\% reduction in labor supply around the time of childbirth, and a 45\% increase in hospital delivery. There is a transient 10\% increase in fertility, but mortality reductions are largest in households receiving transfers after pregnancies began, ruling out selection bias. Mortality effects dissipate rapidly when cash is distributed more than three months from the birth. Mortality reductions are concentrated among households with limited (monetary) consumption gains,  suggesting a trade-off between financial and health investments. </t>
+  </si>
+  <si>
+    <t xml:space="preserve">This paper studies whether risk aversion prevents firms in low and middle-income economies from making profitable but uncertain investments. While economists typically model firms as risk neutral, I posit that this assumption is unlikely to hold for the modal developing-country firm, which is owner-operated, meaning business losses threaten owners' consumption. I develop a model showing how risk aversion can reduce firms’ willingness to experiment with new technologies. I test the model’s predictions within the context of retailers' decision to adopt and sell a new product using two field experiments with over 1,200 Kenyan firms. First, offering firms an insurance contract that creates a mean-preserving contraction of profits increases adoption by 50\%. Second, a temporary supplier returns policy increases post-intervention stocking by 70\%. These persistent effects arise through a reduction in the variance of beliefs, not changes in expected profits. Third, increasing the continuation value of learning expands adoption by 80\%. These results show that a feature of developing economies -- small firms in the presence of incomplete financial markets -- creates a barrier to firm growth. Furthermore, the findings suggest that risk aversion constrains the retail market for new products, harming incentives for companies to introduce goods in developing countries. </t>
+  </si>
+  <si>
+    <t>&lt;b&gt;Job Market Paper&lt;/b&gt; &lt;br&gt; Coverage: &lt;a href="https://blogs.worldbank.org/en/impactevaluations/when-risk-aversion-keeps-firms-small--evidence-from-kenyan-retai0"&gt;World Bank Development Impact&lt;/a&gt;, &lt;a href="https://theeconomicmisfit.com/2026/02/13/can-firm-risk-aversion-undermine-retail-markets-in-developing-countries/"&gt;The Economic Misfit&lt;/a&gt;</t>
+  </si>
+  <si>
+    <t>with Michael Walker, Nick Shankar, Edward Miguel and Dennis Egger &lt;br&gt; Coverage: &lt;a href="https://www.nytimes.com/2025/08/18/health/cash-transfer-kenya-poverty.html"&gt;New York Times&lt;/a&gt;, &lt;a href="https://www.npr.org/2025/08/18/nx-s1-5498591/cash-payments-cut-infant-mortality-in-rural-kenya-by-half"&gt;NPR&lt;/a&gt;, &lt;a href="https://www.theguardian.com/global-development/2025/oct/09/money-direct-cash-transfers-women-rural-kenya-a-new-life"&gt;The Guardian&lt;/a&gt;</t>
   </si>
 </sst>
 </file>
@@ -540,15 +540,15 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A8F856E6-0DAE-4AB0-8DFD-4ED5A926F3C8}">
   <dimension ref="A1:E4"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="8.81640625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="28.83203125" style="1" customWidth="1"/>
-    <col min="2" max="2" width="32.1640625" style="1" customWidth="1"/>
-    <col min="3" max="4" width="38.5" style="1" customWidth="1"/>
-    <col min="5" max="16384" width="8.83203125" style="1"/>
+    <col min="1" max="1" width="28.81640625" style="1" customWidth="1"/>
+    <col min="2" max="2" width="32.1796875" style="1" customWidth="1"/>
+    <col min="3" max="4" width="38.453125" style="1" customWidth="1"/>
+    <col min="5" max="16384" width="8.81640625" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" ht="16" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -562,52 +562,52 @@
         <v>2</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="2" spans="1:5" ht="409.6" x14ac:dyDescent="0.2">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" ht="409.5" x14ac:dyDescent="0.35">
       <c r="A2" s="1" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>4</v>
+        <v>26</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>22</v>
+        <v>25</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="E2" s="1">
         <v>1</v>
       </c>
     </row>
-    <row r="3" spans="1:5" ht="350" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:5" ht="348" x14ac:dyDescent="0.35">
       <c r="A3" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="C3" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="D3" s="2" t="s">
         <v>16</v>
-      </c>
-      <c r="C3" s="1" t="s">
-        <v>26</v>
-      </c>
-      <c r="D3" s="2" t="s">
-        <v>18</v>
       </c>
       <c r="E3" s="1">
         <v>1</v>
       </c>
     </row>
-    <row r="4" spans="1:5" ht="380" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:5" ht="377" x14ac:dyDescent="0.35">
       <c r="A4" s="1" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>5</v>
+        <v>27</v>
       </c>
       <c r="C4" s="1" t="s">
-        <v>27</v>
+        <v>24</v>
       </c>
       <c r="D4" s="2" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="E4" s="1">
         <v>1</v>
@@ -626,15 +626,15 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4634DBF9-2A4B-4BD6-9503-80AC50EBF305}">
   <dimension ref="A1:E2"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="8.81640625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="28.83203125" style="1" customWidth="1"/>
-    <col min="2" max="2" width="32.1640625" style="1" customWidth="1"/>
-    <col min="3" max="4" width="38.5" style="1" customWidth="1"/>
-    <col min="5" max="16384" width="8.83203125" style="1"/>
+    <col min="1" max="1" width="28.81640625" style="1" customWidth="1"/>
+    <col min="2" max="2" width="32.1796875" style="1" customWidth="1"/>
+    <col min="3" max="4" width="38.453125" style="1" customWidth="1"/>
+    <col min="5" max="16384" width="8.81640625" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" ht="16" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -648,21 +648,21 @@
         <v>2</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="2" spans="1:5" ht="335" x14ac:dyDescent="0.2">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" ht="348" x14ac:dyDescent="0.35">
       <c r="A2" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="C2" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="D2" s="2" t="s">
         <v>6</v>
-      </c>
-      <c r="B2" s="1" t="s">
-        <v>17</v>
-      </c>
-      <c r="C2" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="D2" s="2" t="s">
-        <v>8</v>
       </c>
     </row>
   </sheetData>
@@ -676,15 +676,15 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D72C59CF-0C37-4915-9D99-95832D380190}">
   <dimension ref="A1:E4"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="8.81640625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="28.83203125" style="1" customWidth="1"/>
-    <col min="2" max="2" width="32.1640625" style="1" customWidth="1"/>
-    <col min="3" max="4" width="38.5" style="1" customWidth="1"/>
-    <col min="5" max="16384" width="8.83203125" style="1"/>
+    <col min="1" max="1" width="28.81640625" style="1" customWidth="1"/>
+    <col min="2" max="2" width="32.1796875" style="1" customWidth="1"/>
+    <col min="3" max="4" width="38.453125" style="1" customWidth="1"/>
+    <col min="5" max="16384" width="8.81640625" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" ht="16" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -698,37 +698,37 @@
         <v>2</v>
       </c>
       <c r="E1" s="1" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" ht="409.5" x14ac:dyDescent="0.35">
+      <c r="A2" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="B2" s="1" t="s">
         <v>12</v>
       </c>
-    </row>
-    <row r="2" spans="1:5" ht="409.6" x14ac:dyDescent="0.2">
-      <c r="A2" s="1" t="s">
+      <c r="C2" s="1" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" ht="29" x14ac:dyDescent="0.35">
+      <c r="A3" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="B3" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="B2" s="1" t="s">
-        <v>14</v>
-      </c>
-      <c r="C2" s="1" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="3" spans="1:5" ht="32" x14ac:dyDescent="0.2">
-      <c r="A3" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="B3" s="1" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="4" spans="1:5" ht="409.6" x14ac:dyDescent="0.2">
+    </row>
+    <row r="4" spans="1:5" ht="391.5" x14ac:dyDescent="0.35">
       <c r="A4" s="1" t="s">
-        <v>23</v>
+        <v>20</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>24</v>
+        <v>21</v>
       </c>
       <c r="C4" s="1" t="s">
-        <v>25</v>
+        <v>22</v>
       </c>
     </row>
   </sheetData>

</xml_diff>